<commit_message>
Add clickable Meta Ad Library links to filtered ads Excel
Rebuilt sustav_ads_active_gray.xlsx with hyperlinked columns:
- Column K: direct link to ad in Meta Ad Library
- Column L: all ads from the fan page

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/creatives/incoming/2026-09-04_meta-adlib/sustav_ads_active_gray.xlsx
+++ b/creatives/incoming/2026-09-04_meta-adlib/sustav_ads_active_gray.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,6 +29,11 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <color rgb="000563C1"/>
+      <sz val="11"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="3">
@@ -56,9 +61,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -424,20 +430,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:O13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
     <col width="6" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
-    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
     <col width="40" customWidth="1" min="8" max="8"/>
     <col width="50" customWidth="1" min="9" max="9"/>
     <col width="50" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="30" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -448,7 +458,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Spend EU</t>
+          <t>Spend</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -478,12 +488,12 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Формат / угол</t>
+          <t>Формат</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Хук (оригинал)</t>
+          <t>Хук</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
@@ -493,7 +503,27 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
+          <t>🔗 Объявление</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>🔗 Все объявления фанки</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
           <t>Ad ID</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Page ID</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Прелендер</t>
         </is>
       </c>
     </row>
@@ -542,9 +572,20 @@
           <t>$185.45</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>открыть →</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
         <is>
           <t>1402275548427010</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>https://bulgarskabilka.bg/pages/antiparazitna-programa</t>
         </is>
       </c>
     </row>
@@ -593,9 +634,20 @@
           <t>$159.33</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>открыть →</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
         <is>
           <t>28024580067184260</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>https://well-zenvex.top/JcjYjp5V</t>
         </is>
       </c>
     </row>
@@ -644,9 +696,20 @@
           <t>$14.07</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>открыть →</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
         <is>
           <t>1387944109399357</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>https://energy-wellness.top/j2pfzG9L</t>
         </is>
       </c>
     </row>
@@ -695,9 +758,29 @@
           <t>$7.76</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>открыть →</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>все объявления →</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
         <is>
           <t>1689968168903357</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>1107110649151742</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>https://joliae-es.com/</t>
         </is>
       </c>
     </row>
@@ -746,9 +829,29 @@
           <t>$4.57</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>открыть →</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>все объявления →</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
         <is>
           <t>1843505113676346</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>1247081985157348</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>https://belviat.com/products/belviat-detox-sada-s-ricinovym-olejem</t>
         </is>
       </c>
     </row>
@@ -797,9 +900,29 @@
           <t>Я 41 год проработал директором похоронного бюро. Своими руками забальзамировал больше 9 000 человек</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>открыть →</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>все объявления →</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
         <is>
           <t>2152049695738291</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>114434101764341</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>https://purplesandcrate.shop/YJ6Zt9hP; https://purplesandcrate.shop/ZyCgHRmT</t>
         </is>
       </c>
     </row>
@@ -837,24 +960,40 @@
           <t>fhije.com; konbjk.com</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Исповедь холистического ветеринара + история жены</t>
-        </is>
-      </c>
+      <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Είκοσι χρόνια. Χιλιάδες ζώα. Και μια μέρα κατάλαβα ότι οι ίδιοι παράσιτοι που καταστρέφουν το ζώο κατέστρεφαν και τη γυναίκα μου. / Благодарение на анонимен благодетел и неговия фонд „Живот без паразити“ жена ми Елена успя да се излекува.</t>
+          <t>Είκοσι χρόνια. Χιλιάδες ζώα. Και μια μέρα κατάλαβα ότι οι ίδιοι παράσιτοι που καταστρέφουν το ζώο από μέσα κατέστρεφαν και τη γυναίκα μου.</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Двадцать лет. Тысячи животных. И однажды я понял, что те же паразиты, что разрушают животное, разрушали и мою жену. / Благодаря анонимному благотворителю и его фонду «Жизнь без паразитов» моя жена Елена смогла вылечиться</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
+          <t>Двадцать лет. Тысячи животных. И однажды я понял, что те же паразиты, что разрушают животное изнутри, разрушали и мою жену</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>открыть →</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>все объявления →</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
         <is>
           <t>1077131035275955</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>120898664436871</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>https://fhije.com/; https://konbjk.com/</t>
         </is>
       </c>
     </row>
@@ -892,24 +1031,40 @@
           <t>be-terralis.com</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Исповедь судмедэксперта</t>
-        </is>
-      </c>
+      <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Гледах как на 2700 семейства казват „не знаем“. Но истинската причина за смъртта е тайна, която ме принуждаваха да заличавам от всеки акт.</t>
+          <t>Гледах как на 2700 семейства казват „не знаем“. Но истинската причина за смъртта е тайна, която ме принуждаваха да заличавам.</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Я видел, как 2 700 семьям говорят «мы не знаем». Но настоящая причина смерти — тайна, которую меня заставляли стирать из каждого акта</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
+          <t>Я видел, как 2 700 семьям говорят «мы не знаем». Но настоящая причина смерти — тайна, которую меня заставляли стирать</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>открыть →</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>все объявления →</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
         <is>
           <t>2275253056636363</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>1190075947531930</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>https://www.be-terralis.com/blogs/news/actualites-purelis-bg</t>
         </is>
       </c>
     </row>
@@ -958,9 +1113,29 @@
           <t>Жизнь с паразитами может выматывать и держать в тревоге, но правильная информация меняет многое</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>открыть →</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>все объявления →</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
         <is>
           <t>1022825640743734</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>1275510835642489</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>https://info.medivaio.com/2M3vs1TG; https://info.medivaio.com/vQH8JwP8</t>
         </is>
       </c>
     </row>
@@ -995,27 +1170,43 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>sprint-good.com; health-quorag.top; enerlu-nexaic.com</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>Врач-лаборант: три отрицательных анализа</t>
-        </is>
-      </c>
+          <t>sprint-good.com; health-quorag.top</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Три пъти подписах резултата ѝ: отрицателен. На четвъртия тя дойде лично, сложи пред мен трите стари бланки и попита: — Тогава защо с всеки месец ми става по-зле? / Извадих нещо от себе си, което ме кара да повръщам и до сега.</t>
+          <t>Три пъти подписах резултата ѝ: отрицателен. На четвъртия тя дойде лично, сложи пред мен трите стари бланки и попита: — Тогава защо с всеки месец ми става по-зле?</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Трижды я подписала её результат: отрицательный. На четвёртый раз она пришла лично, положила передо мной три старых бланка и спросила: — Тогда почему мне с каждым месяцем всё хуже? / Я вытащила из себя нечто, от воспоминания о чём меня до сих пор тошнит</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
+          <t>Трижды я подписывала её результат: отрицательный. На четвёртый раз она пришла лично, положила передо мной три старых бланка и спросила: — Тогда почему мне с каждым месяцем всё хуже?</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>открыть →</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>все объявления →</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
         <is>
           <t>1939713386725141</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>106163668463882</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>https://sprint-good.com/PZcTCngL; https://health-quorag.top/ffY8JnPZ</t>
         </is>
       </c>
     </row>
@@ -1035,7 +1226,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1045,7 +1236,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Harmonie Santé</t>
+          <t>Salazar 1</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1053,24 +1244,40 @@
           <t>be-terralis.com</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Исповедь судмедэксперта</t>
-        </is>
-      </c>
+      <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Пенсионирах се като съдебен лекар преди шест седмици. 31 години. Над 7 000 тела. И сега ще кажа публично нещо, за което щяха да ме изхвърлят по всяко време.</t>
+          <t>Пенсионирах се като съдебен лекар преди шест седмици. 31 години. Над 7 000 тела.</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Я вышел на пенсию с должности судмедэксперта шесть недель назад. 31 год. Более 7 000 тел. И сейчас скажу публично то, за что меня выгнали бы в любой момент</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>1372531254346812</t>
+          <t>Я вышел на пенсию с должности судмедэксперта шесть недель назад. 31 год. Более 7 000 тел</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>открыть →</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>все объявления →</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>1758635278675667</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>785613974633112</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>https://www.be-terralis.com/blogs/news/actualites-purelis-bg</t>
         </is>
       </c>
     </row>
@@ -1119,13 +1326,56 @@
           <t>Освободите организм от нежеланных паразитов и верните лёгкость и энергию</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>открыть →</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>все объявления →</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
         <is>
           <t>1386869403641882</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>122101336424004321</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>https://corebalance.online/VSQrMXKG</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L5" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L6" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L7" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L8" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K12" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId21"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>